<commit_message>
Added TableS5 + cosmetic changes
</commit_message>
<xml_diff>
--- a/Supplemental Files/Table S1.xlsx
+++ b/Supplemental Files/Table S1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Šimon Pavlů\Desktop\2. Differencial analysis of barley promoterome\Supplement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B050D19E-0EA3-467A-8521-71CFDE3043B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B83BE9AF-9EA8-4FBF-98D1-90B5F9C42EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48,20 +48,41 @@
     <t>4DAGxINF</t>
   </si>
   <si>
-    <t>TableS2 - Number of long and short shifts identified between samples</t>
-  </si>
-  <si>
     <t>short</t>
   </si>
   <si>
     <t>long</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>TableS1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> - Number of long and short shifts identified between samples</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -70,9 +91,26 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -170,7 +208,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -178,6 +216,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
@@ -688,8 +727,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>7</v>
+      <c r="A1" s="7" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -717,7 +756,7 @@
     </row>
     <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" s="5">
         <v>618</v>
@@ -740,7 +779,7 @@
     </row>
     <row r="4" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B4" s="5">
         <v>4939</v>
@@ -762,7 +801,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>